<commit_message>
docs: synchronize PRO2192_Project plan.xlsx with Word report ending strictly on 11/08/2026
</commit_message>
<xml_diff>
--- a/tailieu/PRO2192_Project plan.xlsx
+++ b/tailieu/PRO2192_Project plan.xlsx
@@ -791,7 +791,7 @@
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t>Thiết kế cơ sở dữ liệu quan hệ (ERD 32 bảng), cấu hình Fluent API trong EF Core</t>
+          <t>Thiết kế cơ sở dữ liệu quan hệ (ERD 55 bảng), cấu hình Fluent API trong EF Core</t>
         </is>
       </c>
       <c r="D10" s="9" t="inlineStr">
@@ -2059,7 +2059,7 @@
       </c>
       <c r="F44" s="9" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="G44" s="9" t="inlineStr">
@@ -2096,12 +2096,12 @@
       </c>
       <c r="E45" s="6" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="F45" s="6" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="G45" s="6" t="inlineStr">
@@ -2128,7 +2128,7 @@
       </c>
       <c r="C46" s="9" t="inlineStr">
         <is>
-          <t>Hoàn thiện Báo cáo tốt nghiệp Word (PRO2192), Slide thuyết trình và chuẩn bị bảo vệ</t>
+          <t>Hoàn thiện Báo cáo tốt nghiệp Word (PRO2192), Slide thuyết trình, đóng gói USB bàn giao</t>
         </is>
       </c>
       <c r="D46" s="9" t="inlineStr">
@@ -2138,12 +2138,12 @@
       </c>
       <c r="E46" s="9" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="F46" s="9" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="G46" s="9" t="inlineStr">

</xml_diff>